<commit_message>
Fix python p values
</commit_message>
<xml_diff>
--- a/python/CaseStudy_1/CaseStudy_1/outputs/results/CaseStudy_1_results.xlsx
+++ b/python/CaseStudy_1/CaseStudy_1/outputs/results/CaseStudy_1_results.xlsx
@@ -1701,13 +1701,13 @@
         <v>0.2001128698757735</v>
       </c>
       <c r="E2" t="n">
-        <v>1.266186285081933e-18</v>
+        <v>1.642468918959613e-10</v>
       </c>
       <c r="F2" t="n">
-        <v>1.370517895545833</v>
+        <v>1.356884202431262</v>
       </c>
       <c r="G2" t="n">
-        <v>2.154945931144765</v>
+        <v>2.168579624259336</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -1731,13 +1731,13 @@
         <v>0.0004694940357941142</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0002286061691251302</v>
+        <v>0.0007472694241579085</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.002650327373480022</v>
+        <v>-0.002682314009857343</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0008099445712543761</v>
+        <v>-0.0007779579348770551</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -1761,13 +1761,13 @@
         <v>0.007860148045872805</v>
       </c>
       <c r="E4" t="n">
-        <v>0.003187507546922771</v>
+        <v>0.005570051766146455</v>
       </c>
       <c r="F4" t="n">
-        <v>0.007774375061896075</v>
+        <v>0.007238863046306814</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03858558922802324</v>
+        <v>0.0391211012436125</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -1791,13 +1791,13 @@
         <v>0.0008454978967663197</v>
       </c>
       <c r="E5" t="n">
-        <v>6.996230109484501e-11</v>
+        <v>1.407830752705295e-07</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.007170415686691578</v>
+        <v>-0.007228019472298588</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.003856124833358876</v>
+        <v>-0.003798521047751866</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -1821,13 +1821,13 @@
         <v>47.02894543312258</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4183913842490631</v>
+        <v>0.4243676331404952</v>
       </c>
       <c r="F6" t="n">
-        <v>-130.2315758699673</v>
+        <v>-133.8513636506407</v>
       </c>
       <c r="G6" t="n">
-        <v>54.11850268967207</v>
+        <v>57.7382904703454</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1851,13 +1851,13 @@
         <v>0.07300693936642831</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5290333241045773</v>
+        <v>0.533502140177099</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1890475511048993</v>
+        <v>-0.194666848424648</v>
       </c>
       <c r="G7" t="n">
-        <v>0.09713439245449863</v>
+        <v>0.1027536897742474</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -1881,13 +1881,13 @@
         <v>0.6439711402781584</v>
       </c>
       <c r="E8" t="n">
-        <v>2.628883032767623e-09</v>
+        <v>1.242803417492055e-06</v>
       </c>
       <c r="F8" t="n">
-        <v>2.571553324517899</v>
+        <v>2.521987278687677</v>
       </c>
       <c r="G8" t="n">
-        <v>5.095873808574662</v>
+        <v>5.145439854404883</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
@@ -1911,13 +1911,13 @@
         <v>0.07382882680094055</v>
       </c>
       <c r="E9" t="n">
-        <v>0.33986119911668</v>
+        <v>0.3470160514961801</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.07423668998256061</v>
+        <v>-0.07991924745124823</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2151669931188173</v>
+        <v>0.2208495505875049</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
@@ -1941,13 +1941,13 @@
         <v>1.227757567238736</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5806286652700818</v>
+        <v>0.5844673229707076</v>
       </c>
       <c r="F10" t="n">
-        <v>-3.084655745602748</v>
+        <v>-3.17915545846235</v>
       </c>
       <c r="G10" t="n">
-        <v>1.728065481466126</v>
+        <v>1.822565194325728</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -1971,13 +1971,13 @@
         <v>0.1469216346081419</v>
       </c>
       <c r="E11" t="n">
-        <v>7.490302853562755e-06</v>
+        <v>8.961169890710422e-05</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.9460609891102365</v>
+        <v>-0.9573694531375108</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.370138764346813</v>
+        <v>-0.3588303003195388</v>
       </c>
       <c r="H11" t="b">
         <v>1</v>
@@ -2001,13 +2001,13 @@
         <v>2.26044859478304</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7648521737475424</v>
+        <v>0.7667862481127761</v>
       </c>
       <c r="F12" t="n">
-        <v>-5.106532294858995</v>
+        <v>-5.280517574071167</v>
       </c>
       <c r="G12" t="n">
-        <v>3.754263374498874</v>
+        <v>3.928248653711046</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
@@ -2031,13 +2031,13 @@
         <v>0.1060352714646493</v>
       </c>
       <c r="E13" t="n">
-        <v>5.147845702556687e-09</v>
+        <v>1.714149884685754e-06</v>
       </c>
       <c r="F13" t="n">
-        <v>0.4116667908862169</v>
+        <v>0.4035053240186697</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8273174172094978</v>
+        <v>0.8354788840770451</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>
@@ -2061,13 +2061,13 @@
         <v>15.38974612967395</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1115886425344325</v>
+        <v>0.1203330021854069</v>
       </c>
       <c r="F14" t="n">
-        <v>-54.64986583388973</v>
+        <v>-55.69836949071794</v>
       </c>
       <c r="G14" t="n">
-        <v>5.676830456861538</v>
+        <v>6.725334113689748</v>
       </c>
       <c r="H14" t="b">
         <v>0</v>
@@ -2091,13 +2091,13 @@
         <v>0.5805704949046835</v>
       </c>
       <c r="E15" t="n">
-        <v>4.730141478747253e-11</v>
+        <v>1.177801548125854e-07</v>
       </c>
       <c r="F15" t="n">
-        <v>2.681787038462548</v>
+        <v>2.642232761099883</v>
       </c>
       <c r="G15" t="n">
-        <v>4.957581559462096</v>
+        <v>4.997135836824762</v>
       </c>
       <c r="H15" t="b">
         <v>1</v>
@@ -2121,13 +2121,13 @@
         <v>0.120148270063826</v>
       </c>
       <c r="E16" t="n">
-        <v>2.710111429367325e-08</v>
+        <v>2.699280791115879e-06</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.9034147660313468</v>
+        <v>-0.9116004696460804</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.4324422017715649</v>
+        <v>-0.4242564981568313</v>
       </c>
       <c r="H16" t="b">
         <v>1</v>
@@ -2151,13 +2151,13 @@
         <v>0.09120235041980292</v>
       </c>
       <c r="E17" t="n">
-        <v>3.707160321014081e-11</v>
+        <v>1.054901616861433e-07</v>
       </c>
       <c r="F17" t="n">
-        <v>0.4245806053169425</v>
+        <v>0.4183669876834386</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7820872495733728</v>
+        <v>0.7883008672068768</v>
       </c>
       <c r="H17" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
CS1 with missing data
</commit_message>
<xml_diff>
--- a/python/CaseStudy_1/CaseStudy_1/outputs/results/CaseStudy_1_results.xlsx
+++ b/python/CaseStudy_1/CaseStudy_1/outputs/results/CaseStudy_1_results.xlsx
@@ -452,12 +452,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>65.38 ± 8.27</t>
+          <t>65.30 ± 6.63</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[45.00, 86.00]</t>
+          <t>[49.00, 82.00]</t>
         </is>
       </c>
     </row>
@@ -492,12 +492,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>96.02 ± 11.34</t>
+          <t>96.10 ± 11.15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[73.50, 120.10]</t>
+          <t>[74.00, 119.00]</t>
         </is>
       </c>
     </row>
@@ -512,12 +512,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.75 ± 0.07</t>
+          <t>0.70 ± 0.13</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[0.57, 0.88]</t>
+          <t>[0.39, 0.93]</t>
         </is>
       </c>
     </row>
@@ -532,12 +532,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>36.88 ± 11.44</t>
+          <t>31.95 ± 9.30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[5.00, 61.00]</t>
+          <t>[3.00, 48.00]</t>
         </is>
       </c>
     </row>
@@ -552,12 +552,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>21.63 ± 6.10</t>
+          <t>21.73 ± 6.00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>[8.17, 30.00]</t>
+          <t>[8.00, 30.00]</t>
         </is>
       </c>
     </row>
@@ -592,12 +592,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>426.01 ± 14.80</t>
+          <t>426.25 ± 19.48</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>[402.10, 453.20]</t>
+          <t>[397.00, 460.10]</t>
         </is>
       </c>
     </row>
@@ -632,12 +632,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>350.27 ± 18.06</t>
+          <t>400.63 ± 57.50</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[313.60, 398.10]</t>
+          <t>[292.90, 553.70]</t>
         </is>
       </c>
     </row>
@@ -694,10 +694,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.3276986272214049</v>
+        <v>-0.3207696065048913</v>
       </c>
       <c r="D2" t="n">
-        <v>0.03899761503832627</v>
+        <v>0.04358378460168066</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -715,10 +715,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.1883090182217046</v>
+        <v>0.0287158250175099</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2445652747308571</v>
+        <v>0.8603788229641178</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -736,10 +736,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-0.7100482729789244</v>
+        <v>-0.4422573779878733</v>
       </c>
       <c r="D4" t="n">
-        <v>2.878279572222926e-07</v>
+        <v>0.004271817614390119</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -757,13 +757,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.5058569594093072</v>
+        <v>-0.2063388030970709</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0008686831197336607</v>
+        <v>0.2014546546120567</v>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.2834915929037181</v>
+        <v>-0.2329719477101329</v>
       </c>
       <c r="D6" t="n">
-        <v>0.07628317966422776</v>
+        <v>0.1479770003889512</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -799,10 +799,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.110962650001924</v>
+        <v>-0.1050292290181772</v>
       </c>
       <c r="D7" t="n">
-        <v>0.4954632280323287</v>
+        <v>0.5189355611697632</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -820,10 +820,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.1805939658732494</v>
+        <v>0.07756243706362424</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2647828549380568</v>
+        <v>0.6342807125507927</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -841,10 +841,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.1516306078865655</v>
+        <v>0.1571837430812517</v>
       </c>
       <c r="D9" t="n">
-        <v>0.350302679495509</v>
+        <v>0.3327284916884576</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -862,10 +862,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.5023222042534468</v>
+        <v>0.4264802731085177</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0009569168482815385</v>
+        <v>0.006066038716375244</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -883,13 +883,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.3171137580189982</v>
+        <v>0.2497524343343926</v>
       </c>
       <c r="D11" t="n">
-        <v>0.04617419698504174</v>
+        <v>0.1201293735263728</v>
       </c>
       <c r="E11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -904,10 +904,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.2117487183861192</v>
+        <v>0.1035379429791611</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1896275873430526</v>
+        <v>0.5249204448895113</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -925,10 +925,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.2413211843703935</v>
+        <v>0.1741627171168726</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1335826591951864</v>
+        <v>0.2824580608492747</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.2355355144361428</v>
+        <v>0.2234894746911969</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1434414278887164</v>
+        <v>0.165668484242298</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.02920737342315189</v>
+        <v>0.02920737342315184</v>
       </c>
       <c r="D15" t="n">
         <v>0.8580130044521453</v>
@@ -988,10 +988,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.04637245701105736</v>
+        <v>-0.00844938876332995</v>
       </c>
       <c r="D16" t="n">
-        <v>0.7763046662292736</v>
+        <v>0.9587319186370518</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-0.1695728623476228</v>
+        <v>-0.1695728623476229</v>
       </c>
       <c r="D17" t="n">
         <v>0.2955313155035025</v>
@@ -1030,10 +1030,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-0.3712959149202616</v>
+        <v>-0.3545882105755914</v>
       </c>
       <c r="D18" t="n">
-        <v>0.01833243880399955</v>
+        <v>0.02476783850610207</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -1051,13 +1051,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.3567360902999702</v>
+        <v>0.2220046870708253</v>
       </c>
       <c r="D19" t="n">
-        <v>0.02384787520595973</v>
+        <v>0.1685713198009995</v>
       </c>
       <c r="E19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1072,10 +1072,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.5036108733763326</v>
+        <v>0.5588448209307196</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0009238676796105992</v>
+        <v>0.0001782426447959368</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.2185720769811642</v>
+        <v>0.1620321768304164</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1754221319580761</v>
+        <v>0.3178399955733318</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -1114,10 +1114,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.03544301344759995</v>
+        <v>0.003327431726896316</v>
       </c>
       <c r="D22" t="n">
-        <v>0.8281138531763589</v>
+        <v>0.9837424427446484</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -1135,10 +1135,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-0.2706662992756537</v>
+        <v>-0.242403711075757</v>
       </c>
       <c r="D23" t="n">
-        <v>0.09117025603824867</v>
+        <v>0.131795342246067</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -1156,13 +1156,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-0.3137570217392106</v>
+        <v>-0.2854600331340953</v>
       </c>
       <c r="D24" t="n">
-        <v>0.04866091224574502</v>
+        <v>0.07417742781277253</v>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1177,10 +1177,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-0.3033159685501475</v>
+        <v>-0.2094610707281932</v>
       </c>
       <c r="D25" t="n">
-        <v>0.05709257741631503</v>
+        <v>0.1945673896838412</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -1198,13 +1198,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.4464564182275069</v>
+        <v>0.2259053384273919</v>
       </c>
       <c r="D26" t="n">
-        <v>0.003880347627246363</v>
+        <v>0.1610227829036922</v>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1219,10 +1219,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.193628521063276</v>
+        <v>0.07955126670813464</v>
       </c>
       <c r="D27" t="n">
-        <v>0.2312474467715116</v>
+        <v>0.6255875240590609</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1240,10 +1240,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.3450111807807595</v>
+        <v>0.4031055969784398</v>
       </c>
       <c r="D28" t="n">
-        <v>0.02923629230489992</v>
+        <v>0.009906335836704727</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -1261,10 +1261,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>-0.4596246932145684</v>
+        <v>-0.6513915203479713</v>
       </c>
       <c r="D29" t="n">
-        <v>0.00284806149662708</v>
+        <v>5.31154035994957e-06</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -1282,10 +1282,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>-0.1415952740161406</v>
+        <v>-0.04880456745587317</v>
       </c>
       <c r="D30" t="n">
-        <v>0.3834632425205142</v>
+        <v>0.7648961001572275</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1303,10 +1303,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>-0.468611764659109</v>
+        <v>-0.3434870272649356</v>
       </c>
       <c r="D31" t="n">
-        <v>0.00228989446758346</v>
+        <v>0.03000532623504752</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -1324,10 +1324,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.2784684926214037</v>
+        <v>0.2044633053211565</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0818689175462257</v>
+        <v>0.2056728302539272</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1345,10 +1345,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-0.03613452235338056</v>
+        <v>-0.08945870137830392</v>
       </c>
       <c r="D33" t="n">
-        <v>0.8248120333505894</v>
+        <v>0.5830410856016189</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1366,10 +1366,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-0.2445718510223799</v>
+        <v>-0.2244290541942728</v>
       </c>
       <c r="D34" t="n">
-        <v>0.1282691948378934</v>
+        <v>0.1638503092043211</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1387,10 +1387,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.3301766796318241</v>
+        <v>0.3762486202860814</v>
       </c>
       <c r="D35" t="n">
-        <v>0.03745621950837999</v>
+        <v>0.01671975880815285</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
@@ -1408,10 +1408,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>-0.4627162756001863</v>
+        <v>-0.3435498800882303</v>
       </c>
       <c r="D36" t="n">
-        <v>0.002643905867692089</v>
+        <v>0.02997328637250541</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
@@ -1429,10 +1429,10 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.1227150199789093</v>
+        <v>0.1157156911908309</v>
       </c>
       <c r="D37" t="n">
-        <v>0.4506299369860684</v>
+        <v>0.4770610821920201</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1450,10 +1450,10 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-0.01048902954241881</v>
+        <v>0.02668848959996191</v>
       </c>
       <c r="D38" t="n">
-        <v>0.948781874753659</v>
+        <v>0.8701488690598943</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1471,10 +1471,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>-0.1737427103182844</v>
+        <v>-0.1730353164649613</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2836384645112817</v>
+        <v>0.2856337898742209</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1492,10 +1492,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-0.1777987171943505</v>
+        <v>-0.1256737929599666</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2723730586470292</v>
+        <v>0.4397012408729351</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1513,10 +1513,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>-0.006009928421320895</v>
+        <v>0.006855151701204104</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9706403971100127</v>
+        <v>0.9665135107826465</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1555,10 +1555,10 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>-0.2832343802963874</v>
+        <v>-0.2845210467290931</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0765617563325247</v>
+        <v>0.07517615408809161</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1576,10 +1576,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>-0.1211291587419557</v>
+        <v>-0.1381752605898812</v>
       </c>
       <c r="D44" t="n">
-        <v>0.4565477723353288</v>
+        <v>0.3951721342916746</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1597,10 +1597,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.1851858969803987</v>
+        <v>0.1314399689516148</v>
       </c>
       <c r="D45" t="n">
-        <v>0.2526204065392658</v>
+        <v>0.4188285516109804</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>-0.012792214140414</v>
+        <v>-0.02791488698284272</v>
       </c>
       <c r="D46" t="n">
-        <v>0.9375554634806053</v>
+        <v>0.8642363003757815</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1695,19 +1695,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.762731913345299</v>
+        <v>2.733810686500823</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2001128698757735</v>
+        <v>0.2755661337104445</v>
       </c>
       <c r="E2" t="n">
-        <v>1.642468918959613e-10</v>
+        <v>7.68147362157133e-12</v>
       </c>
       <c r="F2" t="n">
-        <v>1.356884202431262</v>
+        <v>2.174936663849294</v>
       </c>
       <c r="G2" t="n">
-        <v>2.168579624259336</v>
+        <v>3.292684709152352</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -1725,19 +1725,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.001730135972367199</v>
+        <v>-0.004168184582649111</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0004694940357941142</v>
+        <v>0.0005947899755515322</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0007472694241579085</v>
+        <v>3.206129998987174e-08</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.002682314009857343</v>
+        <v>-0.005374474563908481</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0007779579348770551</v>
+        <v>-0.002961894601389739</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -1755,19 +1755,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.02317998214495966</v>
+        <v>0.05484520874341514</v>
       </c>
       <c r="D4" t="n">
-        <v>0.007860148045872805</v>
+        <v>0.01327857418623916</v>
       </c>
       <c r="E4" t="n">
-        <v>0.005570051766146455</v>
+        <v>0.0002057194809773241</v>
       </c>
       <c r="F4" t="n">
-        <v>0.007238863046306814</v>
+        <v>0.02791501209472963</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0391211012436125</v>
+        <v>0.08177540539210065</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -1785,19 +1785,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.005513270260025227</v>
+        <v>-0.006935367739447966</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0008454978967663197</v>
+        <v>0.00175696906993948</v>
       </c>
       <c r="E5" t="n">
-        <v>1.407830752705295e-07</v>
+        <v>0.0003514613978268959</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.007228019472298588</v>
+        <v>-0.01049866617010043</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.003798521047751866</v>
+        <v>-0.003372069308795506</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -1815,19 +1815,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-38.05653659014764</v>
+        <v>-51.65229783499778</v>
       </c>
       <c r="D6" t="n">
-        <v>47.02894543312258</v>
+        <v>27.62387375201347</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4243676331404952</v>
+        <v>0.07067880827543956</v>
       </c>
       <c r="F6" t="n">
-        <v>-133.8513636506407</v>
+        <v>-107.9202873560063</v>
       </c>
       <c r="G6" t="n">
-        <v>57.7382904703454</v>
+        <v>4.615691686010749</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1845,19 +1845,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.04595657932520032</v>
+        <v>-0.01082258620199875</v>
       </c>
       <c r="D7" t="n">
-        <v>0.07300693936642831</v>
+        <v>0.01826804491971371</v>
       </c>
       <c r="E7" t="n">
-        <v>0.533502140177099</v>
+        <v>0.557724346845434</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.194666848424648</v>
+        <v>-0.04803337601879051</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1027536897742474</v>
+        <v>0.02638820361479301</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -1875,19 +1875,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3.83371356654628</v>
+        <v>3.376296480169991</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6439711402781584</v>
+        <v>0.5368855186305516</v>
       </c>
       <c r="E8" t="n">
-        <v>1.242803417492055e-06</v>
+        <v>4.718414773052992e-07</v>
       </c>
       <c r="F8" t="n">
-        <v>2.521987278687677</v>
+        <v>2.282696465650552</v>
       </c>
       <c r="G8" t="n">
-        <v>5.145439854404883</v>
+        <v>4.469896494689431</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
@@ -1905,19 +1905,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.07046515156812835</v>
+        <v>0.04021436050881816</v>
       </c>
       <c r="D9" t="n">
-        <v>0.07382882680094055</v>
+        <v>0.04604025698897464</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3470160514961801</v>
+        <v>0.3889197905811437</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.07991924745124823</v>
+        <v>-0.05356657409349626</v>
       </c>
       <c r="G9" t="n">
-        <v>0.2208495505875049</v>
+        <v>0.1339952951111326</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
@@ -1935,19 +1935,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-0.678295132068311</v>
+        <v>-0.6417933147544401</v>
       </c>
       <c r="D10" t="n">
-        <v>1.227757567238736</v>
+        <v>1.022226427678122</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5844673229707076</v>
+        <v>0.5345648021379222</v>
       </c>
       <c r="F10" t="n">
-        <v>-3.17915545846235</v>
+        <v>-2.724000409858113</v>
       </c>
       <c r="G10" t="n">
-        <v>1.822565194325728</v>
+        <v>1.440413780349233</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -1965,19 +1965,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.6580998767285248</v>
+        <v>-0.455266606089473</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1469216346081419</v>
+        <v>0.1498283456795954</v>
       </c>
       <c r="E11" t="n">
-        <v>8.961169890710422e-05</v>
+        <v>0.004706145008698081</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.9573694531375108</v>
+        <v>-0.7604569591997072</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.3588303003195388</v>
+        <v>-0.1500762529792388</v>
       </c>
       <c r="H11" t="b">
         <v>1</v>
@@ -1995,19 +1995,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.6761344601800605</v>
+        <v>-0.6189476054179561</v>
       </c>
       <c r="D12" t="n">
-        <v>2.26044859478304</v>
+        <v>1.875090348960794</v>
       </c>
       <c r="E12" t="n">
-        <v>0.7667862481127761</v>
+        <v>0.7434836682158715</v>
       </c>
       <c r="F12" t="n">
-        <v>-5.280517574071167</v>
+        <v>-4.438381659216434</v>
       </c>
       <c r="G12" t="n">
-        <v>3.928248653711046</v>
+        <v>3.200486448380522</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
@@ -2025,19 +2025,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.6194921040478574</v>
+        <v>0.6395087019022804</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1060352714646493</v>
+        <v>0.08821795163004084</v>
       </c>
       <c r="E13" t="n">
-        <v>1.714149884685754e-06</v>
+        <v>3.092327812792054e-08</v>
       </c>
       <c r="F13" t="n">
-        <v>0.4035053240186697</v>
+        <v>0.4598146147352998</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8354788840770451</v>
+        <v>0.819202789069261</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>
@@ -2055,22 +2055,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-24.4865176885141</v>
+        <v>-39.83626406086096</v>
       </c>
       <c r="D14" t="n">
-        <v>15.38974612967395</v>
+        <v>12.3967314751085</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1203330021854069</v>
+        <v>0.002765179851064838</v>
       </c>
       <c r="F14" t="n">
-        <v>-55.69836949071794</v>
+        <v>-64.97800079729402</v>
       </c>
       <c r="G14" t="n">
-        <v>6.725334113689748</v>
+        <v>-14.69452732442789</v>
       </c>
       <c r="H14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2085,19 +2085,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3.819684298962322</v>
+        <v>3.378190908223435</v>
       </c>
       <c r="D15" t="n">
-        <v>0.5805704949046835</v>
+        <v>0.4825937831412415</v>
       </c>
       <c r="E15" t="n">
-        <v>1.177801548125854e-07</v>
+        <v>3.282094718886378e-08</v>
       </c>
       <c r="F15" t="n">
-        <v>2.642232761099883</v>
+        <v>2.399445351724223</v>
       </c>
       <c r="G15" t="n">
-        <v>4.997135836824762</v>
+        <v>4.356936464722647</v>
       </c>
       <c r="H15" t="b">
         <v>1</v>
@@ -2115,19 +2115,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.6679284839014559</v>
+        <v>-0.461561249760049</v>
       </c>
       <c r="D16" t="n">
-        <v>0.120148270063826</v>
+        <v>0.1234959243631254</v>
       </c>
       <c r="E16" t="n">
-        <v>2.699280791115879e-06</v>
+        <v>0.0006436733186906978</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.9116004696460804</v>
+        <v>-0.712022593106439</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.4242564981568313</v>
+        <v>-0.2110999064136591</v>
       </c>
       <c r="H16" t="b">
         <v>1</v>
@@ -2145,19 +2145,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.6033339274451577</v>
+        <v>0.627177611815128</v>
       </c>
       <c r="D17" t="n">
-        <v>0.09120235041980292</v>
+        <v>0.07566252085798209</v>
       </c>
       <c r="E17" t="n">
-        <v>1.054901616861433e-07</v>
+        <v>7.246298232408195e-10</v>
       </c>
       <c r="F17" t="n">
-        <v>0.4183669876834386</v>
+        <v>0.4737269071639963</v>
       </c>
       <c r="G17" t="n">
-        <v>0.7883008672068768</v>
+        <v>0.7806283164662596</v>
       </c>
       <c r="H17" t="b">
         <v>1</v>
@@ -2196,7 +2196,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.120226469458207</v>
+        <v>1.122159224626421</v>
       </c>
     </row>
     <row r="3">
@@ -2206,7 +2206,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.047077145488536</v>
+        <v>1.031567982301406</v>
       </c>
     </row>
     <row r="4">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.134707451455411</v>
+        <v>1.095337554489827</v>
       </c>
     </row>
   </sheetData>

</xml_diff>